<commit_message>
Add Impact on KPI to all Incon and MML tables as report v1.7.
Findings sheets rename KPI impact to Impact on KPI. MML suggestion
tables (RIM, scheduling, access/PHY, MIMO combined, 10-site RIM) get a
new column naming Throughput, Accessibility, Drop, HOSR, EN-DC, Latency,
or Interference. v1.6 is kept as history.

Co-authored-by: Mohammad Selim <miles4482@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/5G_NSA_RIM_Type1_RS_MML_10sites_DHK_9Sep26.xlsx
+++ b/5G_NSA_RIM_Type1_RS_MML_10sites_DHK_9Sep26.xlsx
@@ -111,8 +111,71 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -499,7 +562,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -513,1567 +576,1724 @@
     <col width="36" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.9" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Type-1 RIM-RS trial MML  ·  10 sites × 3 cells  ·  DHK dump 8 Sep 2026</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Select the NE in MAE, then copy the MML cell of that row and paste. One MOD per cell. Size=20, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70. SetId=(gNodeBId%10000)*10+(NrDuCellId%10). LST after each cell before RimAlgoSwitch. Do not mix UlIntrfRandomSchSwitch. Inconsistency report v1.4 is unchanged.</t>
+    <row r="2" ht="31" customHeight="1">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>Select the NE in MAE, then copy the MML cell of that row and paste. One MOD per cell. Size=20, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70. SetId=(gNodeBId%10000)*10+(NrDuCellId%10). LST after each cell before RimAlgoSwitch. Do not mix UlIntrfRandomSchSwitch. Inconsistency report v1.4 is unchanged. Impact on KPI column added (v1.7). Inconsistency report v1.6 leftover pack is unchanged in v1.6 file; current report is v1.7.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" s="3" t="n"/>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
+      <c r="A3" s="24" t="n"/>
+      <c r="B3" s="24" t="n"/>
+      <c r="C3" s="24" t="n"/>
+      <c r="D3" s="24" t="n"/>
+      <c r="E3" s="24" t="n"/>
+      <c r="F3" s="24" t="n"/>
+      <c r="G3" s="24" t="n"/>
+      <c r="H3" s="24" t="n"/>
+      <c r="I3" s="24" t="n"/>
+      <c r="J3" s="24" t="n"/>
+      <c r="K3" s="24" t="n"/>
+      <c r="L3" s="24" t="n"/>
     </row>
     <row r="4" ht="33.7" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>SN</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="25" t="inlineStr">
         <is>
           <t>gNodeB Name</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="25" t="inlineStr">
         <is>
           <t>gNodeB ID</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="25" t="inlineStr">
         <is>
           <t>NR DU Cell ID</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="25" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F4" s="26" t="inlineStr">
         <is>
           <t>MML Command (Proposed)</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="26" t="inlineStr">
         <is>
           <t>MO Name</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H4" s="26" t="inlineStr">
         <is>
           <t>RimRsType1SetId</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="26" t="inlineStr">
         <is>
           <t>Live Value (actual in Dump)</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J4" s="26" t="inlineStr">
         <is>
           <t>proposed Parameter Value</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K4" s="26" t="inlineStr">
         <is>
           <t>Purpose/Short Notes</t>
         </is>
       </c>
+      <c r="L4" s="26" t="inlineStr">
+        <is>
+          <t>Impact on KPI</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="71.5" customHeight="1">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>DHDHN35</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n">
+      <c r="C5" s="27" t="n">
         <v>1130258</v>
       </c>
-      <c r="D5" s="6" t="n">
+      <c r="D5" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="E5" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2581, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="n">
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H5" s="27" t="n">
         <v>2581</v>
       </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="I5" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J5" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2581, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN35 (gNodeBId=1130258, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L5" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="71.5" customHeight="1">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="27" t="inlineStr">
         <is>
           <t>DHDHN35</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n">
+      <c r="C6" s="27" t="n">
         <v>1130258</v>
       </c>
-      <c r="D6" s="6" t="n">
+      <c r="D6" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E6" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="E6" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F6" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2582, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="n">
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H6" s="27" t="n">
         <v>2582</v>
       </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="I6" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J6" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2582, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN35 (gNodeBId=1130258, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L6" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="71.5" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>DHDHN35</t>
         </is>
       </c>
-      <c r="C7" s="6" t="n">
+      <c r="C7" s="27" t="n">
         <v>1130258</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="D7" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="E7" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2583, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="n">
+      <c r="G7" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H7" s="27" t="n">
         <v>2583</v>
       </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="I7" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J7" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2583, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K7" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN35 (gNodeBId=1130258, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L7" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="71.5" customHeight="1">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="27" t="inlineStr">
         <is>
           <t>DHDHN10</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n">
+      <c r="C8" s="27" t="n">
         <v>1130236</v>
       </c>
-      <c r="D8" s="6" t="n">
+      <c r="D8" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E8" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="E8" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2361, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n">
+      <c r="G8" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="n">
         <v>2361</v>
       </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="I8" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J8" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2361, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN10 (gNodeBId=1130236, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L8" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="71.5" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>DHDHN10</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n">
+      <c r="C9" s="27" t="n">
         <v>1130236</v>
       </c>
-      <c r="D9" s="6" t="n">
+      <c r="D9" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2362, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="n">
+      <c r="G9" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H9" s="27" t="n">
         <v>2362</v>
       </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="I9" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J9" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2362, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K9" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN10 (gNodeBId=1130236, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L9" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="71.5" customHeight="1">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="B10" s="27" t="inlineStr">
         <is>
           <t>DHDHN10</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n">
+      <c r="C10" s="27" t="n">
         <v>1130236</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="D10" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="E10" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F10" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2363, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="n">
+      <c r="G10" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="n">
         <v>2363</v>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="I10" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J10" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2363, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN10 (gNodeBId=1130236, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L10" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="71.5" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>DHDHN02</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="27" t="n">
         <v>1130228</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="D11" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="E11" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F11" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2281, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="n">
+      <c r="G11" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H11" s="27" t="n">
         <v>2281</v>
       </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="I11" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J11" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2281, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K11" s="6" t="inlineStr">
+      <c r="K11" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN02 (gNodeBId=1130228, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L11" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="71.5" customHeight="1">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="6" t="inlineStr">
+      <c r="B12" s="27" t="inlineStr">
         <is>
           <t>DHDHN02</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n">
+      <c r="C12" s="27" t="n">
         <v>1130228</v>
       </c>
-      <c r="D12" s="6" t="n">
+      <c r="D12" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E12" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="E12" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F12" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2282, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="n">
+      <c r="G12" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H12" s="27" t="n">
         <v>2282</v>
       </c>
-      <c r="I12" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="I12" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J12" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2282, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN02 (gNodeBId=1130228, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L12" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="71.5" customHeight="1">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>DHDHN02</t>
         </is>
       </c>
-      <c r="C13" s="6" t="n">
+      <c r="C13" s="27" t="n">
         <v>1130228</v>
       </c>
-      <c r="D13" s="6" t="n">
+      <c r="D13" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="E13" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F13" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2283, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="n">
+      <c r="G13" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H13" s="27" t="n">
         <v>2283</v>
       </c>
-      <c r="I13" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr">
+      <c r="I13" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J13" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2283, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
+      <c r="K13" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN02 (gNodeBId=1130228, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L13" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="71.5" customHeight="1">
-      <c r="A14" s="6" t="n">
+      <c r="A14" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="6" t="inlineStr">
+      <c r="B14" s="27" t="inlineStr">
         <is>
           <t>DHKLB77</t>
         </is>
       </c>
-      <c r="C14" s="6" t="n">
+      <c r="C14" s="27" t="n">
         <v>1134811</v>
       </c>
-      <c r="D14" s="6" t="n">
+      <c r="D14" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E14" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=48111, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="n">
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H14" s="27" t="n">
         <v>48111</v>
       </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="I14" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J14" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=48111, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K14" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB77 (gNodeBId=1134811, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L14" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="71.5" customHeight="1">
-      <c r="A15" s="6" t="n">
+      <c r="A15" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>DHKLB77</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n">
+      <c r="C15" s="27" t="n">
         <v>1134811</v>
       </c>
-      <c r="D15" s="6" t="n">
+      <c r="D15" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="E15" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=48112, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="n">
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H15" s="27" t="n">
         <v>48112</v>
       </c>
-      <c r="I15" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="I15" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J15" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=48112, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="K15" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB77 (gNodeBId=1134811, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L15" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="71.5" customHeight="1">
-      <c r="A16" s="6" t="n">
+      <c r="A16" s="27" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B16" s="27" t="inlineStr">
         <is>
           <t>DHKLB77</t>
         </is>
       </c>
-      <c r="C16" s="6" t="n">
+      <c r="C16" s="27" t="n">
         <v>1134811</v>
       </c>
-      <c r="D16" s="6" t="n">
+      <c r="D16" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F16" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=48113, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="n">
+      <c r="G16" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H16" s="27" t="n">
         <v>48113</v>
       </c>
-      <c r="I16" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="I16" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J16" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=48113, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="K16" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB77 (gNodeBId=1134811, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L16" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="71.5" customHeight="1">
-      <c r="A17" s="6" t="n">
+      <c r="A17" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>DHDHN27</t>
         </is>
       </c>
-      <c r="C17" s="6" t="n">
+      <c r="C17" s="27" t="n">
         <v>1130251</v>
       </c>
-      <c r="D17" s="6" t="n">
+      <c r="D17" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2511, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="n">
+      <c r="G17" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H17" s="27" t="n">
         <v>2511</v>
       </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="I17" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J17" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2511, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="K17" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN27 (gNodeBId=1130251, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L17" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="71.5" customHeight="1">
-      <c r="A18" s="6" t="n">
+      <c r="A18" s="27" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="27" t="inlineStr">
         <is>
           <t>DHDHN27</t>
         </is>
       </c>
-      <c r="C18" s="6" t="n">
+      <c r="C18" s="27" t="n">
         <v>1130251</v>
       </c>
-      <c r="D18" s="6" t="n">
+      <c r="D18" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F18" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2512, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="n">
+      <c r="G18" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H18" s="27" t="n">
         <v>2512</v>
       </c>
-      <c r="I18" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr">
+      <c r="I18" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J18" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2512, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="K18" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN27 (gNodeBId=1130251, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L18" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="71.5" customHeight="1">
-      <c r="A19" s="6" t="n">
+      <c r="A19" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>DHDHN27</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n">
+      <c r="C19" s="27" t="n">
         <v>1130251</v>
       </c>
-      <c r="D19" s="6" t="n">
+      <c r="D19" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E19" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="E19" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F19" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2513, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="n">
+      <c r="G19" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H19" s="27" t="n">
         <v>2513</v>
       </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
+      <c r="I19" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J19" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2513, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="K19" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN27 (gNodeBId=1130251, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L19" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="71.5" customHeight="1">
-      <c r="A20" s="6" t="n">
+      <c r="A20" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="6" t="inlineStr">
+      <c r="B20" s="27" t="inlineStr">
         <is>
           <t>DHKLB47</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="27" t="n">
         <v>1130803</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="D20" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E20" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="E20" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F20" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=8031, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="n">
+      <c r="G20" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H20" s="27" t="n">
         <v>8031</v>
       </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="I20" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J20" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=8031, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K20" s="6" t="inlineStr">
+      <c r="K20" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB47 (gNodeBId=1130803, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L20" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="71.5" customHeight="1">
-      <c r="A21" s="6" t="n">
+      <c r="A21" s="27" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="6" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>DHKLB47</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n">
+      <c r="C21" s="27" t="n">
         <v>1130803</v>
       </c>
-      <c r="D21" s="6" t="n">
+      <c r="D21" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="E21" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F21" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=8032, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="n">
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H21" s="27" t="n">
         <v>8032</v>
       </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
+      <c r="I21" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J21" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=8032, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K21" s="6" t="inlineStr">
+      <c r="K21" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB47 (gNodeBId=1130803, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L21" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="71.5" customHeight="1">
-      <c r="A22" s="6" t="n">
+      <c r="A22" s="27" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="6" t="inlineStr">
+      <c r="B22" s="27" t="inlineStr">
         <is>
           <t>DHKLB47</t>
         </is>
       </c>
-      <c r="C22" s="6" t="n">
+      <c r="C22" s="27" t="n">
         <v>1130803</v>
       </c>
-      <c r="D22" s="6" t="n">
+      <c r="D22" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E22" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="E22" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F22" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=8033, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="n">
+      <c r="G22" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H22" s="27" t="n">
         <v>8033</v>
       </c>
-      <c r="I22" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J22" s="6" t="inlineStr">
+      <c r="I22" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J22" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=8033, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
+      <c r="K22" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB47 (gNodeBId=1130803, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L22" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="71.5" customHeight="1">
-      <c r="A23" s="6" t="n">
+      <c r="A23" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="6" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>DHDHN37</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n">
+      <c r="C23" s="27" t="n">
         <v>1130260</v>
       </c>
-      <c r="D23" s="6" t="n">
+      <c r="D23" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F23" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2601, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="n">
+      <c r="G23" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H23" s="27" t="n">
         <v>2601</v>
       </c>
-      <c r="I23" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J23" s="6" t="inlineStr">
+      <c r="I23" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J23" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2601, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K23" s="6" t="inlineStr">
+      <c r="K23" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN37 (gNodeBId=1130260, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L23" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="71.5" customHeight="1">
-      <c r="A24" s="6" t="n">
+      <c r="A24" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="6" t="inlineStr">
+      <c r="B24" s="27" t="inlineStr">
         <is>
           <t>DHDHN37</t>
         </is>
       </c>
-      <c r="C24" s="6" t="n">
+      <c r="C24" s="27" t="n">
         <v>1130260</v>
       </c>
-      <c r="D24" s="6" t="n">
+      <c r="D24" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="E24" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F24" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2602, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="n">
+      <c r="G24" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H24" s="27" t="n">
         <v>2602</v>
       </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J24" s="6" t="inlineStr">
+      <c r="I24" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J24" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2602, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K24" s="6" t="inlineStr">
+      <c r="K24" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN37 (gNodeBId=1130260, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L24" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="71.5" customHeight="1">
-      <c r="A25" s="6" t="n">
+      <c r="A25" s="27" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>DHDHN37</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n">
+      <c r="C25" s="27" t="n">
         <v>1130260</v>
       </c>
-      <c r="D25" s="6" t="n">
+      <c r="D25" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="E25" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F25" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2603, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="n">
+      <c r="G25" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H25" s="27" t="n">
         <v>2603</v>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J25" s="6" t="inlineStr">
+      <c r="I25" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J25" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2603, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K25" s="6" t="inlineStr">
+      <c r="K25" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN37 (gNodeBId=1130260, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L25" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="71.5" customHeight="1">
-      <c r="A26" s="6" t="n">
+      <c r="A26" s="27" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="27" t="inlineStr">
         <is>
           <t>DHDHN40</t>
         </is>
       </c>
-      <c r="C26" s="6" t="n">
+      <c r="C26" s="27" t="n">
         <v>1130263</v>
       </c>
-      <c r="D26" s="6" t="n">
+      <c r="D26" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E26" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="E26" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F26" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2631, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="n">
+      <c r="G26" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="n">
         <v>2631</v>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J26" s="6" t="inlineStr">
+      <c r="I26" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J26" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2631, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K26" s="6" t="inlineStr">
+      <c r="K26" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN40 (gNodeBId=1130263, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L26" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="71.5" customHeight="1">
-      <c r="A27" s="6" t="n">
+      <c r="A27" s="27" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="6" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>DHDHN40</t>
         </is>
       </c>
-      <c r="C27" s="6" t="n">
+      <c r="C27" s="27" t="n">
         <v>1130263</v>
       </c>
-      <c r="D27" s="6" t="n">
+      <c r="D27" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F27" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2632, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="n">
+      <c r="G27" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="n">
         <v>2632</v>
       </c>
-      <c r="I27" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J27" s="6" t="inlineStr">
+      <c r="I27" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J27" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2632, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K27" s="6" t="inlineStr">
+      <c r="K27" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN40 (gNodeBId=1130263, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L27" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="71.5" customHeight="1">
-      <c r="A28" s="6" t="n">
+      <c r="A28" s="27" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="6" t="inlineStr">
+      <c r="B28" s="27" t="inlineStr">
         <is>
           <t>DHDHN40</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n">
+      <c r="C28" s="27" t="n">
         <v>1130263</v>
       </c>
-      <c r="D28" s="6" t="n">
+      <c r="D28" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E28" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="E28" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2633, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="n">
+      <c r="G28" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="n">
         <v>2633</v>
       </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J28" s="6" t="inlineStr">
+      <c r="I28" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J28" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2633, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K28" s="6" t="inlineStr">
+      <c r="K28" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN40 (gNodeBId=1130263, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L28" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="71.5" customHeight="1">
-      <c r="A29" s="6" t="n">
+      <c r="A29" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>DHKLB66</t>
         </is>
       </c>
-      <c r="C29" s="6" t="n">
+      <c r="C29" s="27" t="n">
         <v>1134551</v>
       </c>
-      <c r="D29" s="6" t="n">
+      <c r="D29" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E29" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="E29" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F29" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=45511, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="n">
+      <c r="G29" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="n">
         <v>45511</v>
       </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr">
+      <c r="I29" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J29" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=45511, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K29" s="6" t="inlineStr">
+      <c r="K29" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB66 (gNodeBId=1134551, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L29" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="71.5" customHeight="1">
-      <c r="A30" s="6" t="n">
+      <c r="A30" s="27" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="6" t="inlineStr">
+      <c r="B30" s="27" t="inlineStr">
         <is>
           <t>DHKLB66</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n">
+      <c r="C30" s="27" t="n">
         <v>1134551</v>
       </c>
-      <c r="D30" s="6" t="n">
+      <c r="D30" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E30" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
+      <c r="E30" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F30" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=45512, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="n">
+      <c r="G30" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="n">
         <v>45512</v>
       </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J30" s="6" t="inlineStr">
+      <c r="I30" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J30" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=45512, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K30" s="6" t="inlineStr">
+      <c r="K30" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB66 (gNodeBId=1134551, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L30" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="71.5" customHeight="1">
-      <c r="A31" s="6" t="n">
+      <c r="A31" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="6" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>DHKLB66</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n">
+      <c r="C31" s="27" t="n">
         <v>1134551</v>
       </c>
-      <c r="D31" s="6" t="n">
+      <c r="D31" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="E31" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F31" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=45513, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="n">
+      <c r="G31" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="n">
         <v>45513</v>
       </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J31" s="6" t="inlineStr">
+      <c r="I31" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J31" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=45513, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K31" s="6" t="inlineStr">
+      <c r="K31" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHKLB66 (gNodeBId=1134551, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L31" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="71.5" customHeight="1">
-      <c r="A32" s="6" t="n">
+      <c r="A32" s="27" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="6" t="inlineStr">
+      <c r="B32" s="27" t="inlineStr">
         <is>
           <t>DHDHN05</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n">
+      <c r="C32" s="27" t="n">
         <v>1130231</v>
       </c>
-      <c r="D32" s="6" t="n">
+      <c r="D32" s="27" t="n">
         <v>101</v>
       </c>
-      <c r="E32" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F32" s="6" t="inlineStr">
+      <c r="E32" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F32" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=101, RimRsType1SetIdSize=20, RimRsType1SetId=2311, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="n">
+      <c r="G32" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="n">
         <v>2311</v>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J32" s="6" t="inlineStr">
+      <c r="I32" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J32" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2311, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K32" s="6" t="inlineStr">
+      <c r="K32" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN05 (gNodeBId=1130231, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L32" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="71.5" customHeight="1">
-      <c r="A33" s="6" t="n">
+      <c r="A33" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="6" t="inlineStr">
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>DHDHN05</t>
         </is>
       </c>
-      <c r="C33" s="6" t="n">
+      <c r="C33" s="27" t="n">
         <v>1130231</v>
       </c>
-      <c r="D33" s="6" t="n">
+      <c r="D33" s="27" t="n">
         <v>102</v>
       </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="E33" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F33" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=102, RimRsType1SetIdSize=20, RimRsType1SetId=2312, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="n">
+      <c r="G33" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="n">
         <v>2312</v>
       </c>
-      <c r="I33" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J33" s="6" t="inlineStr">
+      <c r="I33" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J33" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2312, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K33" s="6" t="inlineStr">
+      <c r="K33" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN05 (gNodeBId=1130231, 32T32R, n41 40 MHz, 8:2 SS54).</t>
         </is>
       </c>
+      <c r="L33" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="71.5" customHeight="1">
-      <c r="A34" s="6" t="n">
+      <c r="A34" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="6" t="inlineStr">
+      <c r="B34" s="27" t="inlineStr">
         <is>
           <t>DHDHN05</t>
         </is>
       </c>
-      <c r="C34" s="6" t="n">
+      <c r="C34" s="27" t="n">
         <v>1130231</v>
       </c>
-      <c r="D34" s="6" t="n">
+      <c r="D34" s="27" t="n">
         <v>103</v>
       </c>
-      <c r="E34" s="7" t="inlineStr">
-        <is>
-          <t>Enable</t>
-        </is>
-      </c>
-      <c r="F34" s="6" t="inlineStr">
+      <c r="E34" s="28" t="inlineStr">
+        <is>
+          <t>Enable</t>
+        </is>
+      </c>
+      <c r="F34" s="27" t="inlineStr">
         <is>
           <t>MOD NRDUCELLRIMCONFIG: NrDuCellId=103, RimRsType1SetIdSize=20, RimRsType1SetId=2313, RimRsFreqCandNum=FREQ_NUM_2, RimRsType1SeqCandNum=SEQ_NUM_8, RimRsType1ScidForIs0=0, RimRsType1ScidForIs1=10, RimRsType1ScidForIs2=20, RimRsType1ScidForIs3=30, RimRsType1ScidForIs4=40, RimRsType1ScidForIs5=50, RimRsType1ScidForIs6=60, RimRsType1ScidForIs7=70;</t>
         </is>
       </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>NRDUCellRimConfig</t>
-        </is>
-      </c>
-      <c r="H34" s="6" t="n">
+      <c r="G34" s="27" t="inlineStr">
+        <is>
+          <t>NRDUCellRimConfig</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="n">
         <v>2313</v>
       </c>
-      <c r="I34" s="6" t="inlineStr">
-        <is>
-          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
-        </is>
-      </c>
-      <c r="J34" s="6" t="inlineStr">
+      <c r="I34" s="27" t="inlineStr">
+        <is>
+          <t>Size=255 / SetId=4294967295 / Freq=NULL / Seq=NULL / Scid=4294967295</t>
+        </is>
+      </c>
+      <c r="J34" s="27" t="inlineStr">
         <is>
           <t>Size=20, SetId=2313, FREQ_NUM_2, SEQ_NUM_8, Scid 0/10/20/30/40/50/60/70</t>
         </is>
       </c>
-      <c r="K34" s="6" t="inlineStr">
+      <c r="K34" s="27" t="inlineStr">
         <is>
           <t>Paste on NE DHDHN05 (gNodeBId=1130231, 32T32R, n41 40 MHz, 8:2 SS54).</t>
+        </is>
+      </c>
+      <c r="L34" s="27" t="inlineStr">
+        <is>
+          <t>UL Throughput · UL Interference (IoT) · Accessibility (RACH under remote interference) · Drop if Type-1 RS SetId collides</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:K34"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>